<commit_message>
Versão 2.0 - OCR silencioso e extração completa de fornecedores
</commit_message>
<xml_diff>
--- a/saida_teste_notas.xlsx
+++ b/saida_teste_notas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -608,6 +608,32 @@
       </c>
       <c r="C13" s="3" t="n">
         <v>558</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DVC COMERCIO E SERVICOS LTDA</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>2858</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DVC COMERCIO E SERVICOS LTDA</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>2858</v>
       </c>
     </row>
   </sheetData>
@@ -621,7 +647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -797,103 +823,134 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n"/>
-      <c r="B10" s="1" t="n"/>
-      <c r="C10" s="1" t="n"/>
-      <c r="D10" s="1" t="n"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DVC COMERCIO E SERVICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>5716</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Fornecedor</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Total Geral (Todos os Meses)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Quantidade de Notas</t>
-        </is>
-      </c>
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="1" t="n"/>
+      <c r="C11" s="1" t="n"/>
+      <c r="D11" s="1" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HARDWARE AUTOMACAO E TECNOLOGIA LTDA</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>10842.8</v>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>4</v>
+          <t>Fornecedor</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Total Geral (Todos os Meses)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Quantidade de Notas</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>JPBG RAPIDEX COMERCIAL LTDA</t>
+          <t>HARDWARE AUTOMACAO E TECNOLOGIA LTDA</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>3974</v>
+        <v>10842.8</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>R C DOS SANTOS GONCALVES DISTRIBUICAO E SERVICOS LTDA</t>
+          <t>DVC COMERCIO E SERVICOS LTDA</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>2990</v>
+        <v>5716</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ALFAMAR COMERCIO TELEFONIA E ACESSORIOS LTDA</t>
+          <t>JPBG RAPIDEX COMERCIAL LTDA</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>2638</v>
+        <v>3974</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>114 TECH GOLD COMERCIO E SERVIÇO DE INFORMATICA LTDA</t>
+          <t>R C DOS SANTOS GONCALVES DISTRIBUICAO E SERVICOS LTDA</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>2088</v>
+        <v>2990</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>ALFAMAR COMERCIO TELEFONIA E ACESSORIOS LTDA</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>2638</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>114 TECH GOLD COMERCIO E SERVIÇO DE INFORMATICA LTDA</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>2088</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>CICEROANTONIOMENDESBITTAR 00847519759</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B19" s="3" t="n">
         <v>817</v>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C19" s="4" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>